<commit_message>
Fix formula row references in budget calculator
- FOT sheet B4-B7: НДФЛ/СВ rates now point to correct rows (B28-B31) instead of direction toggles (B19-B22)
- Season avg formula: B42,B43 (летние/зимние месяцы) instead of B32,B33
- Estimate sheet: overhead->B35, profit->B36/B37, НДС->B26
- P&L sheet: НДС->B26, УСН->B27, back-office->B38, management->B39

Co-authored-by: kpetlin21-bot <kpetlin21-bot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/budget/output/Калькулятор бюджета ЖК.xlsx
+++ b/budget/output/Калькулятор бюджета ЖК.xlsx
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="B4" s="20">
-        <f>'📋 Параметры'!B19</f>
+        <f>'📋 Параметры'!B28</f>
         <v/>
       </c>
       <c r="C4" s="10" t="inlineStr"/>
@@ -1447,7 +1447,7 @@
         </is>
       </c>
       <c r="B5" s="20">
-        <f>'📋 Параметры'!B20</f>
+        <f>'📋 Параметры'!B29</f>
         <v/>
       </c>
       <c r="C5" s="10" t="inlineStr"/>
@@ -1459,7 +1459,7 @@
         </is>
       </c>
       <c r="B6" s="20">
-        <f>'📋 Параметры'!B21</f>
+        <f>'📋 Параметры'!B30</f>
         <v/>
       </c>
       <c r="C6" s="10" t="inlineStr"/>
@@ -1471,7 +1471,7 @@
         </is>
       </c>
       <c r="B7" s="20">
-        <f>'📋 Параметры'!B22</f>
+        <f>'📋 Параметры'!B31</f>
         <v/>
       </c>
       <c r="C7" s="10" t="inlineStr"/>
@@ -2377,7 +2377,7 @@
       <c r="G41" s="47" t="n"/>
       <c r="H41" s="47" t="n"/>
       <c r="I41" s="48">
-        <f>(I39*'📋 Параметры'!B32+J40*'📋 Параметры'!B33)/12</f>
+        <f>(I39*'📋 Параметры'!B42+J40*'📋 Параметры'!B43)/12</f>
         <v/>
       </c>
     </row>
@@ -2498,7 +2498,7 @@
         <v>0</v>
       </c>
       <c r="D6" s="25">
-        <f>(B6*'📋 Параметры'!B32+C6*'📋 Параметры'!B33)/12</f>
+        <f>(B6*'📋 Параметры'!B42+C6*'📋 Параметры'!B43)/12</f>
         <v/>
       </c>
       <c r="E6" s="10" t="inlineStr"/>
@@ -2516,7 +2516,7 @@
         <v>0</v>
       </c>
       <c r="D7" s="25">
-        <f>(B7*'📋 Параметры'!B32+C7*'📋 Параметры'!B33)/12</f>
+        <f>(B7*'📋 Параметры'!B42+C7*'📋 Параметры'!B43)/12</f>
         <v/>
       </c>
       <c r="E7" s="10" t="inlineStr"/>
@@ -2534,7 +2534,7 @@
         <v>0</v>
       </c>
       <c r="D8" s="25">
-        <f>(B8*'📋 Параметры'!B32+C8*'📋 Параметры'!B33)/12</f>
+        <f>(B8*'📋 Параметры'!B42+C8*'📋 Параметры'!B43)/12</f>
         <v/>
       </c>
       <c r="E8" s="10" t="inlineStr"/>
@@ -2552,7 +2552,7 @@
         <v>0</v>
       </c>
       <c r="D9" s="25">
-        <f>(B9*'📋 Параметры'!B32+C9*'📋 Параметры'!B33)/12</f>
+        <f>(B9*'📋 Параметры'!B42+C9*'📋 Параметры'!B43)/12</f>
         <v/>
       </c>
       <c r="E9" s="10" t="inlineStr"/>
@@ -2601,7 +2601,7 @@
         <v>20000</v>
       </c>
       <c r="D13" s="25">
-        <f>(B13*'📋 Параметры'!B32+C13*'📋 Параметры'!B33)/12</f>
+        <f>(B13*'📋 Параметры'!B42+C13*'📋 Параметры'!B43)/12</f>
         <v/>
       </c>
       <c r="E13" s="10" t="inlineStr"/>
@@ -2619,7 +2619,7 @@
         <v>30000</v>
       </c>
       <c r="D14" s="25">
-        <f>(B14*'📋 Параметры'!B32+C14*'📋 Параметры'!B33)/12</f>
+        <f>(B14*'📋 Параметры'!B42+C14*'📋 Параметры'!B43)/12</f>
         <v/>
       </c>
       <c r="E14" s="10" t="inlineStr"/>
@@ -2637,7 +2637,7 @@
         <v>5000</v>
       </c>
       <c r="D15" s="25">
-        <f>(B15*'📋 Параметры'!B32+C15*'📋 Параметры'!B33)/12</f>
+        <f>(B15*'📋 Параметры'!B42+C15*'📋 Параметры'!B43)/12</f>
         <v/>
       </c>
       <c r="E15" s="10" t="inlineStr"/>
@@ -2655,7 +2655,7 @@
         <v>5000</v>
       </c>
       <c r="D16" s="25">
-        <f>(B16*'📋 Параметры'!B32+C16*'📋 Параметры'!B33)/12</f>
+        <f>(B16*'📋 Параметры'!B42+C16*'📋 Параметры'!B43)/12</f>
         <v/>
       </c>
       <c r="E16" s="10" t="inlineStr"/>
@@ -2673,7 +2673,7 @@
         <v>4000</v>
       </c>
       <c r="D17" s="25">
-        <f>(B17*'📋 Параметры'!B32+C17*'📋 Параметры'!B33)/12</f>
+        <f>(B17*'📋 Параметры'!B42+C17*'📋 Параметры'!B43)/12</f>
         <v/>
       </c>
       <c r="E17" s="10" t="inlineStr"/>
@@ -2687,7 +2687,7 @@
       <c r="B18" s="11" t="n"/>
       <c r="C18" s="11" t="n"/>
       <c r="D18" s="25">
-        <f>(B18*'📋 Параметры'!B32+C18*'📋 Параметры'!B33)/12</f>
+        <f>(B18*'📋 Параметры'!B42+C18*'📋 Параметры'!B43)/12</f>
         <v/>
       </c>
       <c r="E18" s="10" t="inlineStr"/>
@@ -2701,7 +2701,7 @@
       <c r="B19" s="11" t="n"/>
       <c r="C19" s="11" t="n"/>
       <c r="D19" s="25">
-        <f>(B19*'📋 Параметры'!B32+C19*'📋 Параметры'!B33)/12</f>
+        <f>(B19*'📋 Параметры'!B42+C19*'📋 Параметры'!B43)/12</f>
         <v/>
       </c>
       <c r="E19" s="10" t="inlineStr"/>
@@ -2781,11 +2781,11 @@
       <c r="B26" s="10" t="n"/>
       <c r="C26" s="10" t="n"/>
       <c r="D26" s="25">
-        <f>D23*'📋 Параметры'!B27</f>
+        <f>D23*'📋 Параметры'!B35</f>
         <v/>
       </c>
       <c r="E26" s="61">
-        <f>'📋 Параметры'!B27</f>
+        <f>'📋 Параметры'!B35</f>
         <v/>
       </c>
     </row>
@@ -2798,7 +2798,7 @@
       <c r="B27" s="10" t="n"/>
       <c r="C27" s="10" t="n"/>
       <c r="D27" s="25">
-        <f>D23*'📋 Параметры'!B28</f>
+        <f>D23*'📋 Параметры'!B37</f>
         <v/>
       </c>
       <c r="E27" s="61">
@@ -2815,7 +2815,7 @@
       <c r="B28" s="10" t="n"/>
       <c r="C28" s="10" t="n"/>
       <c r="D28" s="25">
-        <f>D23*'📋 Параметры'!B28*'📋 Параметры'!B24</f>
+        <f>D23*'📋 Параметры'!B36*'📋 Параметры'!B32</f>
         <v/>
       </c>
       <c r="E28" s="61" t="inlineStr">
@@ -2847,7 +2847,7 @@
       <c r="B30" s="47" t="n"/>
       <c r="C30" s="47" t="n"/>
       <c r="D30" s="25">
-        <f>D29*'📋 Параметры'!B18</f>
+        <f>D29*'📋 Параметры'!B26</f>
         <v/>
       </c>
       <c r="E30" s="47" t="n"/>
@@ -2914,7 +2914,7 @@
       <c r="B36" s="44" t="n"/>
       <c r="C36" s="44" t="n"/>
       <c r="D36" s="27">
-        <f>D31-D23-D30-D23*'📋 Параметры'!B28*'📋 Параметры'!B24</f>
+        <f>D31-D23-D30-D23*'📋 Параметры'!B36*'📋 Параметры'!B32</f>
         <v/>
       </c>
       <c r="E36" s="44" t="n"/>
@@ -3934,51 +3934,51 @@
         </is>
       </c>
       <c r="B25" s="25">
-        <f>B9*'📋 Параметры'!B29</f>
+        <f>B9*'📋 Параметры'!B38</f>
         <v/>
       </c>
       <c r="C25" s="25">
-        <f>C9*'📋 Параметры'!B29</f>
+        <f>C9*'📋 Параметры'!B38</f>
         <v/>
       </c>
       <c r="D25" s="25">
-        <f>D9*'📋 Параметры'!B29</f>
+        <f>D9*'📋 Параметры'!B38</f>
         <v/>
       </c>
       <c r="E25" s="25">
-        <f>E9*'📋 Параметры'!B29</f>
+        <f>E9*'📋 Параметры'!B38</f>
         <v/>
       </c>
       <c r="F25" s="25">
-        <f>F9*'📋 Параметры'!B29</f>
+        <f>F9*'📋 Параметры'!B38</f>
         <v/>
       </c>
       <c r="G25" s="25">
-        <f>G9*'📋 Параметры'!B29</f>
+        <f>G9*'📋 Параметры'!B38</f>
         <v/>
       </c>
       <c r="H25" s="25">
-        <f>H9*'📋 Параметры'!B29</f>
+        <f>H9*'📋 Параметры'!B38</f>
         <v/>
       </c>
       <c r="I25" s="25">
-        <f>I9*'📋 Параметры'!B29</f>
+        <f>I9*'📋 Параметры'!B38</f>
         <v/>
       </c>
       <c r="J25" s="25">
-        <f>J9*'📋 Параметры'!B29</f>
+        <f>J9*'📋 Параметры'!B38</f>
         <v/>
       </c>
       <c r="K25" s="25">
-        <f>K9*'📋 Параметры'!B29</f>
+        <f>K9*'📋 Параметры'!B38</f>
         <v/>
       </c>
       <c r="L25" s="25">
-        <f>L9*'📋 Параметры'!B29</f>
+        <f>L9*'📋 Параметры'!B38</f>
         <v/>
       </c>
       <c r="M25" s="25">
-        <f>M9*'📋 Параметры'!B29</f>
+        <f>M9*'📋 Параметры'!B38</f>
         <v/>
       </c>
       <c r="N25" s="25">
@@ -3993,51 +3993,51 @@
         </is>
       </c>
       <c r="B26" s="25">
-        <f>B9*'📋 Параметры'!B30</f>
+        <f>B9*'📋 Параметры'!B39</f>
         <v/>
       </c>
       <c r="C26" s="25">
-        <f>C9*'📋 Параметры'!B30</f>
+        <f>C9*'📋 Параметры'!B39</f>
         <v/>
       </c>
       <c r="D26" s="25">
-        <f>D9*'📋 Параметры'!B30</f>
+        <f>D9*'📋 Параметры'!B39</f>
         <v/>
       </c>
       <c r="E26" s="25">
-        <f>E9*'📋 Параметры'!B30</f>
+        <f>E9*'📋 Параметры'!B39</f>
         <v/>
       </c>
       <c r="F26" s="25">
-        <f>F9*'📋 Параметры'!B30</f>
+        <f>F9*'📋 Параметры'!B39</f>
         <v/>
       </c>
       <c r="G26" s="25">
-        <f>G9*'📋 Параметры'!B30</f>
+        <f>G9*'📋 Параметры'!B39</f>
         <v/>
       </c>
       <c r="H26" s="25">
-        <f>H9*'📋 Параметры'!B30</f>
+        <f>H9*'📋 Параметры'!B39</f>
         <v/>
       </c>
       <c r="I26" s="25">
-        <f>I9*'📋 Параметры'!B30</f>
+        <f>I9*'📋 Параметры'!B39</f>
         <v/>
       </c>
       <c r="J26" s="25">
-        <f>J9*'📋 Параметры'!B30</f>
+        <f>J9*'📋 Параметры'!B39</f>
         <v/>
       </c>
       <c r="K26" s="25">
-        <f>K9*'📋 Параметры'!B30</f>
+        <f>K9*'📋 Параметры'!B39</f>
         <v/>
       </c>
       <c r="L26" s="25">
-        <f>L9*'📋 Параметры'!B30</f>
+        <f>L9*'📋 Параметры'!B39</f>
         <v/>
       </c>
       <c r="M26" s="25">
-        <f>M9*'📋 Параметры'!B30</f>
+        <f>M9*'📋 Параметры'!B39</f>
         <v/>
       </c>
       <c r="N26" s="25">
@@ -4296,51 +4296,51 @@
         </is>
       </c>
       <c r="B33" s="25">
-        <f>B9*'📋 Параметры'!B18</f>
+        <f>B9*'📋 Параметры'!B26</f>
         <v/>
       </c>
       <c r="C33" s="25">
-        <f>C9*'📋 Параметры'!B18</f>
+        <f>C9*'📋 Параметры'!B26</f>
         <v/>
       </c>
       <c r="D33" s="25">
-        <f>D9*'📋 Параметры'!B18</f>
+        <f>D9*'📋 Параметры'!B26</f>
         <v/>
       </c>
       <c r="E33" s="25">
-        <f>E9*'📋 Параметры'!B18</f>
+        <f>E9*'📋 Параметры'!B26</f>
         <v/>
       </c>
       <c r="F33" s="25">
-        <f>F9*'📋 Параметры'!B18</f>
+        <f>F9*'📋 Параметры'!B26</f>
         <v/>
       </c>
       <c r="G33" s="25">
-        <f>G9*'📋 Параметры'!B18</f>
+        <f>G9*'📋 Параметры'!B26</f>
         <v/>
       </c>
       <c r="H33" s="25">
-        <f>H9*'📋 Параметры'!B18</f>
+        <f>H9*'📋 Параметры'!B26</f>
         <v/>
       </c>
       <c r="I33" s="25">
-        <f>I9*'📋 Параметры'!B18</f>
+        <f>I9*'📋 Параметры'!B26</f>
         <v/>
       </c>
       <c r="J33" s="25">
-        <f>J9*'📋 Параметры'!B18</f>
+        <f>J9*'📋 Параметры'!B26</f>
         <v/>
       </c>
       <c r="K33" s="25">
-        <f>K9*'📋 Параметры'!B18</f>
+        <f>K9*'📋 Параметры'!B26</f>
         <v/>
       </c>
       <c r="L33" s="25">
-        <f>L9*'📋 Параметры'!B18</f>
+        <f>L9*'📋 Параметры'!B26</f>
         <v/>
       </c>
       <c r="M33" s="25">
-        <f>M9*'📋 Параметры'!B18</f>
+        <f>M9*'📋 Параметры'!B26</f>
         <v/>
       </c>
       <c r="N33" s="25">
@@ -4355,51 +4355,51 @@
         </is>
       </c>
       <c r="B34" s="25">
-        <f>B9*'📋 Параметры'!B19</f>
+        <f>B9*'📋 Параметры'!B27</f>
         <v/>
       </c>
       <c r="C34" s="25">
-        <f>C9*'📋 Параметры'!B19</f>
+        <f>C9*'📋 Параметры'!B27</f>
         <v/>
       </c>
       <c r="D34" s="25">
-        <f>D9*'📋 Параметры'!B19</f>
+        <f>D9*'📋 Параметры'!B27</f>
         <v/>
       </c>
       <c r="E34" s="25">
-        <f>E9*'📋 Параметры'!B19</f>
+        <f>E9*'📋 Параметры'!B27</f>
         <v/>
       </c>
       <c r="F34" s="25">
-        <f>F9*'📋 Параметры'!B19</f>
+        <f>F9*'📋 Параметры'!B27</f>
         <v/>
       </c>
       <c r="G34" s="25">
-        <f>G9*'📋 Параметры'!B19</f>
+        <f>G9*'📋 Параметры'!B27</f>
         <v/>
       </c>
       <c r="H34" s="25">
-        <f>H9*'📋 Параметры'!B19</f>
+        <f>H9*'📋 Параметры'!B27</f>
         <v/>
       </c>
       <c r="I34" s="25">
-        <f>I9*'📋 Параметры'!B19</f>
+        <f>I9*'📋 Параметры'!B27</f>
         <v/>
       </c>
       <c r="J34" s="25">
-        <f>J9*'📋 Параметры'!B19</f>
+        <f>J9*'📋 Параметры'!B27</f>
         <v/>
       </c>
       <c r="K34" s="25">
-        <f>K9*'📋 Параметры'!B19</f>
+        <f>K9*'📋 Параметры'!B27</f>
         <v/>
       </c>
       <c r="L34" s="25">
-        <f>L9*'📋 Параметры'!B19</f>
+        <f>L9*'📋 Параметры'!B27</f>
         <v/>
       </c>
       <c r="M34" s="25">
-        <f>M9*'📋 Параметры'!B19</f>
+        <f>M9*'📋 Параметры'!B27</f>
         <v/>
       </c>
       <c r="N34" s="25">

</xml_diff>